<commit_message>
perf(orchestrator): add concurrent domain processing with ThreadPoolExecutor
Implemented 3-phase concurrent processing pipeline:
- Phase 1: Concurrent domain collection from Google search and scoring
- Phase 2: Batch domain probing to optimize access patterns
- Phase 3: Parallel domain processing with proper synchronization

Key improvements:
- Added process_companies_concurrent() method with ThreadPoolExecutor
- Implemented batch_probe_domains() for efficient access pattern discovery
- Enhanced global state management with proper cleanup and error handling
- Added domain deduplication to prevent redundant processing
- Integrated with CLI for seamless concurrent processing

🤖 Generated with [Claude Code](https://claude.ai/code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,51 +448,51 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>speedy fuels</t>
+          <t xml:space="preserve">petrol rete </t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>speedyfuels.co.uk</t>
+          <t>bpetrol.it</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>hello@speedyfuels.co.uk</t>
+          <t>info@bpetrol.it</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>speedy fuels</t>
+          <t xml:space="preserve">petrol rete </t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>speedyfuels.co.uk</t>
+          <t>bpetrol.it</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>datamanager@speedyfuels.co.uk</t>
+          <t>info@pec.b-petrol.it</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">henan xinlianxin fertilizer </t>
+          <t xml:space="preserve">petrol rete </t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>worldfertilizer.com</t>
+          <t>bpetrol.it</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>enquiries@worldfertilizer.com</t>
+          <t>info@b-petrol.it</t>
         </is>
       </c>
     </row>
@@ -509,24 +509,143 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>support@worldfertilizer.com</t>
+          <t>enquiries@worldfertilizer.com</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t xml:space="preserve">henan xinlianxin fertilizer </t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>worldfertilizer.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>support@worldfertilizer.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Synsol</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>synsol.ch</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>info@synsol.ch</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>euro dam jas doo</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>eurodamjas.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>euro.dam@bih.net.ba</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>speedy fuels</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>speedyfuels.co.uk</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>hello@speedyfuels.co.uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>speedy fuels</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>speedyfuels.co.uk</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>datamanager@speedyfuels.co.uk</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>walter schmidt chemie gmbh</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>walter-schmidt-chemie.de</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>info@walter-schmidt-chemie.de</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>daf trucks</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>daf.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>rutger.kerstiens@daftrucks.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>daf trucks</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>daf.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>dataprotectionofficer@daftrucks.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
I give up - check Surrender_review, will start over with right architecture from the start...
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,106 +444,141 @@
           <t>Email</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>walter schmidt chemie gmbh</t>
+          <t>Synsol</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>walter-schmidt-chemie.de</t>
+          <t>synsol.ch</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>info@walter-schmidt-chemie.de</t>
+          <t>info@synsol.ch</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>async_extraction</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">henan xinlianxin fertilizer </t>
+          <t>walter schmidt chemie gmbh</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>worldfertilizer.com</t>
+          <t>walter-schmidt-chemie.de</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>support@worldfertilizer.com</t>
+          <t>datenschutz@schmidt-zement.de</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>async_extraction</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">henan xinlianxin fertilizer </t>
+          <t>walter schmidt chemie gmbh</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>worldfertilizer.com</t>
+          <t>walter-schmidt-chemie.de</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>enquiries@worldfertilizer.com</t>
+          <t>datenschutz@walter-schmidt-chemie.de</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>async_extraction</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>daf trucks</t>
+          <t>walter schmidt chemie gmbh</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>daf.com</t>
+          <t>walter-schmidt-chemie.de</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>rutger.kerstiens@daftrucks.com</t>
+          <t>info@walter-schmidt-chemie.de</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>async_extraction</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">petrol rete </t>
+          <t>daf trucks</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bpetrol.it</t>
+          <t>daf.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>info@pec.b-petrol.it</t>
+          <t>dataprotectionofficer@daftrucks.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>async_extraction</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">petrol rete </t>
+          <t>daf trucks</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>bpetrol.it</t>
+          <t>daf.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>info@bpetrol.it</t>
+          <t>rutger.kerstiens@daftrucks.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>async_extraction</t>
         </is>
       </c>
     </row>
@@ -555,80 +590,39 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>bpetrol.it</t>
+          <t>alvolante.it</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>info@b-petrol.it</t>
+          <t>info@alvolante.it</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>async_extraction</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>euro dam jas doo</t>
+          <t xml:space="preserve">mitsui toatsu chemicals </t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>eurodamjas.com</t>
+          <t>jp.mitsuichemicals.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>euro.dam@bih.net.ba</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Synsol</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>synsol.ch</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>info@synsol.ch</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>speedy fuels</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>speedyfuels.co.uk</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>datamanager@speedyfuels.co.uk</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>speedy fuels</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>speedyfuels.co.uk</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>hello@speedyfuels.co.uk</t>
+          <t>information@mcs.mitsui-chem.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>async_extraction</t>
         </is>
       </c>
     </row>

</xml_diff>